<commit_message>
Fix Kontrak Ampas Kedelai.xlsx: remove invalid theme color ref, add docProps so Excel opens without repair prompt
</commit_message>
<xml_diff>
--- a/Kontrak Ampas Kedelai.xlsx
+++ b/Kontrak Ampas Kedelai.xlsx
@@ -4,7 +4,7 @@
   <sheets>
     <sheet name="Kontrak Ampas Kedelai" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -19,7 +19,6 @@
   <fonts count="2">
     <font>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -2193,7 +2192,7 @@
     <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="C2:101" error="Masukkan tanggal yang valid (DD/MM/YYYY)." errorTitle="Tanggal Mulai" promptTitle="Tanggal Mulai" prompt="Format DD/MM/YYYY.">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="D2:D101" error="Tanggal Berakhir tidak boleh lebih kecil dari Tanggal Mulai." errorTitle="Tanggal Berakhir" promptTitle="Tanggal Berakhir" prompt="Harus &gt;= Tanggal Mulai (DD/MM/YYYY).">
+    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="D2:D101" error="Tanggal Berakhir tidak boleh lebih kecil dari Tanggal Mulai." errorTitle="Tanggal Berakhir" promptTitle="Tanggal Berakhir" prompt="Harus lebih besar atau sama dengan Tanggal Mulai (DD/MM/YYYY).">
       <formula1>C2</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="E2:101" error="Jumlah Ampas per Hari harus lebih besar dari 0." errorTitle="Jumlah Ampas" promptTitle="Jumlah Ampas per Hari (Kg)" prompt="Isi angka lebih besar dari 0.">

</xml_diff>

<commit_message>
Fix malformed dataValidation sqref (A2:101 -> A2:A101) causing Excel repair prompt
</commit_message>
<xml_diff>
--- a/Kontrak Ampas Kedelai.xlsx
+++ b/Kontrak Ampas Kedelai.xlsx
@@ -2183,22 +2183,22 @@
     </row>
   </sheetData>
   <dataValidations count="6">
-    <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="A2:101" error="Nomor Kontrak tidak boleh kosong." errorTitle="Nomor Kontrak" promptTitle="Nomor Kontrak" prompt="Wajib diisi.">
+    <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="A2:A101" error="Nomor Kontrak tidak boleh kosong." errorTitle="Nomor Kontrak" promptTitle="Nomor Kontrak" prompt="Wajib diisi.">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="B2:101" error="Nama tidak boleh kosong." errorTitle="Nama" promptTitle="Nama" prompt="Wajib diisi.">
+    <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="B2:B101" error="Nama tidak boleh kosong." errorTitle="Nama" promptTitle="Nama" prompt="Wajib diisi.">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="C2:101" error="Masukkan tanggal yang valid (DD/MM/YYYY)." errorTitle="Tanggal Mulai" promptTitle="Tanggal Mulai" prompt="Format DD/MM/YYYY.">
+    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="C2:C101" error="Masukkan tanggal yang valid (DD/MM/YYYY)." errorTitle="Tanggal Mulai" promptTitle="Tanggal Mulai" prompt="Format DD/MM/YYYY.">
       <formula1>1</formula1>
     </dataValidation>
     <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="D2:D101" error="Tanggal Berakhir tidak boleh lebih kecil dari Tanggal Mulai." errorTitle="Tanggal Berakhir" promptTitle="Tanggal Berakhir" prompt="Harus lebih besar atau sama dengan Tanggal Mulai (DD/MM/YYYY).">
       <formula1>C2</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="E2:101" error="Jumlah Ampas per Hari harus lebih besar dari 0." errorTitle="Jumlah Ampas" promptTitle="Jumlah Ampas per Hari (Kg)" prompt="Isi angka lebih besar dari 0.">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="E2:E101" error="Jumlah Ampas per Hari harus lebih besar dari 0." errorTitle="Jumlah Ampas" promptTitle="Jumlah Ampas per Hari (Kg)" prompt="Isi angka lebih besar dari 0.">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="F2:101" error="Harga Kontrak Keseluruhan harus lebih besar dari 0." errorTitle="Harga Kontrak" promptTitle="Harga Kontrak Keseluruhan (Rp)" prompt="Isi angka lebih besar dari 0.">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="F2:F101" error="Harga Kontrak Keseluruhan harus lebih besar dari 0." errorTitle="Harga Kontrak" promptTitle="Harga Kontrak Keseluruhan (Rp)" prompt="Isi angka lebih besar dari 0.">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Remove non-list data validations that triggered Excel repair; formulas still enforce empty output on incomplete data
</commit_message>
<xml_diff>
--- a/Kontrak Ampas Kedelai.xlsx
+++ b/Kontrak Ampas Kedelai.xlsx
@@ -2182,26 +2182,6 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="A2:A101" error="Nomor Kontrak tidak boleh kosong." errorTitle="Nomor Kontrak" promptTitle="Nomor Kontrak" prompt="Wajib diisi.">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="B2:B101" error="Nama tidak boleh kosong." errorTitle="Nama" promptTitle="Nama" prompt="Wajib diisi.">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="C2:C101" error="Masukkan tanggal yang valid (DD/MM/YYYY)." errorTitle="Tanggal Mulai" promptTitle="Tanggal Mulai" prompt="Format DD/MM/YYYY.">
-      <formula1>1</formula1>
-    </dataValidation>
-    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="D2:D101" error="Tanggal Berakhir tidak boleh lebih kecil dari Tanggal Mulai." errorTitle="Tanggal Berakhir" promptTitle="Tanggal Berakhir" prompt="Harus lebih besar atau sama dengan Tanggal Mulai (DD/MM/YYYY).">
-      <formula1>C2</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="E2:E101" error="Jumlah Ampas per Hari harus lebih besar dari 0." errorTitle="Jumlah Ampas" promptTitle="Jumlah Ampas per Hari (Kg)" prompt="Isi angka lebih besar dari 0.">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="F2:F101" error="Harga Kontrak Keseluruhan harus lebih besar dari 0." errorTitle="Harga Kontrak" promptTitle="Harga Kontrak Keseluruhan (Rp)" prompt="Isi angka lebih besar dari 0.">
-      <formula1>0</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>